<commit_message>
added the status column
</commit_message>
<xml_diff>
--- a/custom_import_template/static/xls/import_template.xlsx
+++ b/custom_import_template/static/xls/import_template.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J2"/>
+  <dimension ref="A1:K2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -448,6 +448,7 @@
     <col width="20" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
     <col width="15" customWidth="1" min="10" max="10"/>
+    <col width="15" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -501,6 +502,11 @@
           <t>Date of Birth</t>
         </is>
       </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Status (Import)</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -551,6 +557,11 @@
       <c r="J2" t="inlineStr">
         <is>
           <t>1953-10-18</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Active</t>
         </is>
       </c>
     </row>

</xml_diff>